<commit_message>
feat: Enhance Docker configuration and improve application features
- Removed temporary Excel file and updated docker-compose.yml to include new environment variables for Supabase and Stripe.
- Enhanced next.config.js to support CORS for development and production environments.
- Updated API routes for better error handling and added CORS support.
- Improved user interface with new components for video backgrounds and enhanced reservation modals.
- Updated project data with accurate specifications and improved download functionality for project documents.
</commit_message>
<xml_diff>
--- a/bedrijfunits_opslagboxen.xlsx
+++ b/bedrijfunits_opslagboxen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vireshkewalbansing/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vireshkewalbansing/Repos/unity-units-clone/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A4E9F2-B1C3-814A-93F1-C392C157B759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{793B626D-967C-4C46-9975-D6BD31982166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bedrijfspand" sheetId="1" r:id="rId1"/>
@@ -588,78 +588,6 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -732,6 +660,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -747,11 +681,77 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -765,14 +765,14 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1166,80 +1166,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.3">
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="65" t="s">
+      <c r="C1" s="40"/>
+      <c r="D1" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="66" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="66"/>
-      <c r="O2" s="66"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
       <c r="P2" s="3"/>
     </row>
     <row r="3" spans="1:23" ht="19" x14ac:dyDescent="0.25">
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="67" t="s">
+      <c r="C3" s="40"/>
+      <c r="D3" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
-      <c r="L3" s="67"/>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="43"/>
+      <c r="K3" s="43"/>
+      <c r="L3" s="43"/>
+      <c r="M3" s="43"/>
+      <c r="N3" s="43"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="64"/>
-      <c r="D4" s="68">
+      <c r="C4" s="40"/>
+      <c r="D4" s="44">
         <v>45762</v>
       </c>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="68"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="44"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="44"/>
+      <c r="N4" s="44"/>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="B5" s="2"/>
@@ -1247,142 +1247,142 @@
       <c r="S5" s="2"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="B6" s="88" t="s">
+      <c r="B6" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="89"/>
-      <c r="D6" s="89"/>
-      <c r="E6" s="89"/>
-      <c r="F6" s="89"/>
-      <c r="G6" s="89"/>
-      <c r="H6" s="89"/>
-      <c r="I6" s="89"/>
-      <c r="J6" s="89"/>
-      <c r="K6" s="89"/>
-      <c r="L6" s="90"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="67"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="68"/>
       <c r="M6" s="8"/>
     </row>
     <row r="7" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="40"/>
-      <c r="C7" s="78" t="s">
+      <c r="B7" s="79"/>
+      <c r="C7" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="79"/>
-      <c r="E7" s="79"/>
-      <c r="F7" s="79"/>
-      <c r="G7" s="79"/>
-      <c r="H7" s="80"/>
-      <c r="I7" s="87"/>
-      <c r="J7" s="69" t="s">
+      <c r="D7" s="55"/>
+      <c r="E7" s="55"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="56"/>
+      <c r="I7" s="63"/>
+      <c r="J7" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="70"/>
-      <c r="L7" s="70"/>
-      <c r="M7" s="70"/>
-      <c r="N7" s="70"/>
-      <c r="O7" s="71"/>
-      <c r="P7" s="50"/>
+      <c r="K7" s="46"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="46"/>
+      <c r="N7" s="46"/>
+      <c r="O7" s="47"/>
+      <c r="P7" s="64"/>
       <c r="Q7" s="34" t="s">
         <v>21</v>
       </c>
       <c r="R7" s="35"/>
-      <c r="S7" s="40"/>
+      <c r="S7" s="79"/>
       <c r="U7" s="34" t="s">
         <v>22</v>
       </c>
       <c r="V7" s="35"/>
-      <c r="W7" s="40" t="s">
+      <c r="W7" s="79" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="41"/>
-      <c r="C8" s="81"/>
-      <c r="D8" s="82"/>
-      <c r="E8" s="82"/>
-      <c r="F8" s="82"/>
-      <c r="G8" s="82"/>
-      <c r="H8" s="83"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="72"/>
-      <c r="K8" s="73"/>
-      <c r="L8" s="73"/>
-      <c r="M8" s="73"/>
-      <c r="N8" s="73"/>
-      <c r="O8" s="74"/>
-      <c r="P8" s="50"/>
+      <c r="B8" s="80"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="48"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="49"/>
+      <c r="N8" s="49"/>
+      <c r="O8" s="50"/>
+      <c r="P8" s="64"/>
       <c r="Q8" s="36"/>
       <c r="R8" s="37"/>
-      <c r="S8" s="41"/>
+      <c r="S8" s="80"/>
       <c r="U8" s="36"/>
       <c r="V8" s="37"/>
-      <c r="W8" s="41"/>
+      <c r="W8" s="80"/>
     </row>
     <row r="9" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="42"/>
-      <c r="C9" s="84"/>
-      <c r="D9" s="85"/>
-      <c r="E9" s="85"/>
-      <c r="F9" s="85"/>
-      <c r="G9" s="85"/>
-      <c r="H9" s="86"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="75"/>
-      <c r="K9" s="76"/>
-      <c r="L9" s="76"/>
-      <c r="M9" s="76"/>
-      <c r="N9" s="76"/>
-      <c r="O9" s="77"/>
-      <c r="P9" s="50"/>
+      <c r="B9" s="81"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="62"/>
+      <c r="I9" s="64"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="52"/>
+      <c r="L9" s="52"/>
+      <c r="M9" s="52"/>
+      <c r="N9" s="52"/>
+      <c r="O9" s="53"/>
+      <c r="P9" s="64"/>
       <c r="Q9" s="38"/>
       <c r="R9" s="39"/>
-      <c r="S9" s="42"/>
+      <c r="S9" s="81"/>
       <c r="U9" s="38"/>
       <c r="V9" s="39"/>
-      <c r="W9" s="42"/>
+      <c r="W9" s="81"/>
     </row>
     <row r="10" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="45" t="s">
+      <c r="B10" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="60" t="s">
+      <c r="C10" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="61"/>
-      <c r="E10" s="52" t="s">
+      <c r="D10" s="92"/>
+      <c r="E10" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="F10" s="53"/>
-      <c r="G10" s="52" t="s">
+      <c r="F10" s="86"/>
+      <c r="G10" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="H10" s="53"/>
-      <c r="I10" s="50"/>
-      <c r="J10" s="56" t="s">
+      <c r="H10" s="86"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="89" t="s">
         <v>0</v>
       </c>
-      <c r="K10" s="57"/>
-      <c r="L10" s="56" t="s">
+      <c r="K10" s="90"/>
+      <c r="L10" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="M10" s="57"/>
-      <c r="N10" s="56" t="s">
+      <c r="M10" s="90"/>
+      <c r="N10" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="O10" s="57"/>
-      <c r="P10" s="50"/>
-      <c r="Q10" s="43" t="s">
+      <c r="O10" s="90"/>
+      <c r="P10" s="64"/>
+      <c r="Q10" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="R10" s="44"/>
-      <c r="S10" s="45" t="s">
+      <c r="R10" s="74"/>
+      <c r="S10" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="U10" s="43" t="s">
+      <c r="U10" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="V10" s="44"/>
-      <c r="W10" s="45" t="s">
+      <c r="V10" s="74"/>
+      <c r="W10" s="82" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1390,46 +1390,46 @@
       <c r="A11" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="91" t="s">
+      <c r="B11" s="83"/>
+      <c r="C11" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="92"/>
-      <c r="E11" s="54" t="s">
+      <c r="D11" s="70"/>
+      <c r="E11" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="55"/>
-      <c r="G11" s="54" t="s">
+      <c r="F11" s="88"/>
+      <c r="G11" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H11" s="55"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="58" t="s">
+      <c r="H11" s="88"/>
+      <c r="I11" s="64"/>
+      <c r="J11" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="K11" s="59"/>
-      <c r="L11" s="58" t="s">
+      <c r="K11" s="78"/>
+      <c r="L11" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="M11" s="59"/>
-      <c r="N11" s="58" t="s">
+      <c r="M11" s="78"/>
+      <c r="N11" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="O11" s="59"/>
-      <c r="P11" s="50"/>
-      <c r="Q11" s="48" t="s">
+      <c r="O11" s="78"/>
+      <c r="P11" s="64"/>
+      <c r="Q11" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="R11" s="49"/>
-      <c r="S11" s="46"/>
-      <c r="U11" s="48" t="s">
+      <c r="R11" s="76"/>
+      <c r="S11" s="83"/>
+      <c r="U11" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="V11" s="49"/>
-      <c r="W11" s="46"/>
+      <c r="V11" s="76"/>
+      <c r="W11" s="83"/>
     </row>
     <row r="12" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="47"/>
+      <c r="B12" s="84"/>
       <c r="C12" s="1" t="s">
         <v>4</v>
       </c>
@@ -1448,7 +1448,7 @@
       <c r="H12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I12" s="50"/>
+      <c r="I12" s="64"/>
       <c r="J12" s="1" t="s">
         <v>4</v>
       </c>
@@ -1467,21 +1467,21 @@
       <c r="O12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="P12" s="50"/>
+      <c r="P12" s="64"/>
       <c r="Q12" s="5" t="s">
         <v>4</v>
       </c>
       <c r="R12" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="S12" s="47"/>
+      <c r="S12" s="84"/>
       <c r="U12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="V12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="W12" s="47"/>
+      <c r="W12" s="84"/>
     </row>
     <row r="13" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7">
@@ -1500,7 +1500,7 @@
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
-      <c r="I13" s="50"/>
+      <c r="I13" s="64"/>
       <c r="J13" s="4" t="s">
         <v>18</v>
       </c>
@@ -1517,7 +1517,7 @@
       <c r="O13" s="4">
         <v>44.9</v>
       </c>
-      <c r="P13" s="50"/>
+      <c r="P13" s="64"/>
       <c r="Q13" s="6">
         <f>SUM(C13+L13+N13)</f>
         <v>153.4</v>
@@ -1557,7 +1557,7 @@
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
-      <c r="I14" s="51"/>
+      <c r="I14" s="65"/>
       <c r="J14" s="4" t="s">
         <v>18</v>
       </c>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
-      <c r="P14" s="51"/>
+      <c r="P14" s="65"/>
       <c r="Q14" s="6">
         <f>SUM(C14+L14)</f>
         <v>101.2</v>
@@ -5718,7 +5718,7 @@
       <c r="R93" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="S93" s="40"/>
+      <c r="S93" s="79"/>
     </row>
     <row r="94" spans="1:23" x14ac:dyDescent="0.2">
       <c r="B94" s="17" t="s">
@@ -5737,15 +5737,15 @@
       <c r="M94" s="13"/>
       <c r="N94" s="13"/>
       <c r="O94" s="18"/>
-      <c r="Q94" s="62">
+      <c r="Q94" s="71">
         <f>SUM(Q13:Q91)</f>
         <v>9699.4999999999982</v>
       </c>
-      <c r="R94" s="62">
+      <c r="R94" s="71">
         <f>SUM(R13:R91)</f>
         <v>8964.8999999999978</v>
       </c>
-      <c r="S94" s="41"/>
+      <c r="S94" s="80"/>
       <c r="U94" s="7">
         <f>(SUM(U13:U91))</f>
         <v>20241730</v>
@@ -5766,31 +5766,17 @@
       <c r="M95" s="11"/>
       <c r="N95" s="11"/>
       <c r="O95" s="12"/>
-      <c r="Q95" s="63"/>
-      <c r="R95" s="63"/>
-      <c r="S95" s="42"/>
+      <c r="Q95" s="72"/>
+      <c r="R95" s="72"/>
+      <c r="S95" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="Q7:R9"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D1:L1"/>
-    <mergeCell ref="D2:O2"/>
-    <mergeCell ref="D3:N3"/>
-    <mergeCell ref="D4:N4"/>
-    <mergeCell ref="J7:O9"/>
-    <mergeCell ref="C7:H9"/>
-    <mergeCell ref="I7:I14"/>
-    <mergeCell ref="B6:L6"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="Q94:Q95"/>
-    <mergeCell ref="R94:R95"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="U7:V9"/>
+    <mergeCell ref="W7:W9"/>
+    <mergeCell ref="U10:V10"/>
+    <mergeCell ref="W10:W12"/>
+    <mergeCell ref="U11:V11"/>
     <mergeCell ref="S93:S95"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="S7:S9"/>
@@ -5807,11 +5793,25 @@
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="C10:D10"/>
-    <mergeCell ref="U7:V9"/>
-    <mergeCell ref="W7:W9"/>
-    <mergeCell ref="U10:V10"/>
-    <mergeCell ref="W10:W12"/>
-    <mergeCell ref="U11:V11"/>
+    <mergeCell ref="Q94:Q95"/>
+    <mergeCell ref="R94:R95"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="Q7:R9"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D1:L1"/>
+    <mergeCell ref="D2:O2"/>
+    <mergeCell ref="D3:N3"/>
+    <mergeCell ref="D4:N4"/>
+    <mergeCell ref="J7:O9"/>
+    <mergeCell ref="C7:H9"/>
+    <mergeCell ref="I7:I14"/>
+    <mergeCell ref="B6:L6"/>
+    <mergeCell ref="C11:D11"/>
   </mergeCells>
   <conditionalFormatting sqref="W10:W91">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Ja">
@@ -5867,47 +5867,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="93" t="s">
+      <c r="C1" s="40"/>
+      <c r="D1" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
-      <c r="J1" s="93"/>
-      <c r="K1" s="93"/>
-      <c r="L1" s="93"/>
-      <c r="M1" s="93"/>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="93"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="94"/>
+      <c r="J1" s="94"/>
+      <c r="K1" s="94"/>
+      <c r="L1" s="94"/>
+      <c r="M1" s="94"/>
+      <c r="N1" s="94"/>
+      <c r="O1" s="94"/>
+      <c r="P1" s="94"/>
     </row>
     <row r="2" spans="1:16" ht="38.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="94" t="s">
+      <c r="B2" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
-      <c r="L2" s="94"/>
-      <c r="M2" s="94"/>
-      <c r="N2" s="94"/>
-      <c r="O2" s="94"/>
-      <c r="P2" s="94"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="93"/>
+      <c r="L2" s="93"/>
+      <c r="M2" s="93"/>
+      <c r="N2" s="93"/>
+      <c r="O2" s="93"/>
+      <c r="P2" s="93"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="83" t="s">
         <v>28</v>
       </c>
       <c r="C3" s="95" t="s">
@@ -5932,7 +5932,7 @@
         <v>7</v>
       </c>
       <c r="O3" s="98"/>
-      <c r="P3" s="99" t="s">
+      <c r="P3" s="101" t="s">
         <v>3</v>
       </c>
     </row>
@@ -5940,33 +5940,33 @@
       <c r="A4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="54" t="s">
+      <c r="B4" s="83"/>
+      <c r="C4" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="55"/>
-      <c r="E4" s="54" t="s">
+      <c r="D4" s="88"/>
+      <c r="E4" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="55"/>
-      <c r="G4" s="54" t="s">
+      <c r="F4" s="88"/>
+      <c r="G4" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="55"/>
+      <c r="H4" s="88"/>
       <c r="I4" s="20"/>
-      <c r="J4" s="100" t="s">
+      <c r="J4" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="101"/>
+      <c r="K4" s="100"/>
       <c r="M4" s="2"/>
-      <c r="N4" s="48" t="s">
+      <c r="N4" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="O4" s="49"/>
-      <c r="P4" s="99"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="101"/>
     </row>
     <row r="5" spans="1:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="B5" s="47"/>
+      <c r="B5" s="84"/>
       <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
@@ -7448,47 +7448,47 @@
     </row>
     <row r="44" spans="1:16" ht="33.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="1:16" ht="24" x14ac:dyDescent="0.3">
-      <c r="B46" s="64" t="s">
+      <c r="B46" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C46" s="64"/>
-      <c r="D46" s="93" t="s">
+      <c r="C46" s="40"/>
+      <c r="D46" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="E46" s="93"/>
-      <c r="F46" s="93"/>
-      <c r="G46" s="93"/>
-      <c r="H46" s="93"/>
-      <c r="I46" s="93"/>
-      <c r="J46" s="93"/>
-      <c r="K46" s="93"/>
-      <c r="L46" s="93"/>
-      <c r="M46" s="93"/>
-      <c r="N46" s="93"/>
-      <c r="O46" s="93"/>
-      <c r="P46" s="93"/>
+      <c r="E46" s="94"/>
+      <c r="F46" s="94"/>
+      <c r="G46" s="94"/>
+      <c r="H46" s="94"/>
+      <c r="I46" s="94"/>
+      <c r="J46" s="94"/>
+      <c r="K46" s="94"/>
+      <c r="L46" s="94"/>
+      <c r="M46" s="94"/>
+      <c r="N46" s="94"/>
+      <c r="O46" s="94"/>
+      <c r="P46" s="94"/>
     </row>
     <row r="47" spans="1:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B47" s="94" t="s">
+      <c r="B47" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="C47" s="94"/>
-      <c r="D47" s="94"/>
-      <c r="E47" s="94"/>
-      <c r="F47" s="94"/>
-      <c r="G47" s="94"/>
-      <c r="H47" s="94"/>
-      <c r="I47" s="94"/>
-      <c r="J47" s="94"/>
-      <c r="K47" s="94"/>
-      <c r="L47" s="94"/>
-      <c r="M47" s="94"/>
-      <c r="N47" s="94"/>
-      <c r="O47" s="94"/>
-      <c r="P47" s="94"/>
+      <c r="C47" s="93"/>
+      <c r="D47" s="93"/>
+      <c r="E47" s="93"/>
+      <c r="F47" s="93"/>
+      <c r="G47" s="93"/>
+      <c r="H47" s="93"/>
+      <c r="I47" s="93"/>
+      <c r="J47" s="93"/>
+      <c r="K47" s="93"/>
+      <c r="L47" s="93"/>
+      <c r="M47" s="93"/>
+      <c r="N47" s="93"/>
+      <c r="O47" s="93"/>
+      <c r="P47" s="93"/>
     </row>
     <row r="48" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B48" s="46" t="s">
+      <c r="B48" s="83" t="s">
         <v>28</v>
       </c>
       <c r="C48" s="95" t="s">
@@ -7513,38 +7513,38 @@
         <v>7</v>
       </c>
       <c r="O48" s="98"/>
-      <c r="P48" s="99" t="s">
+      <c r="P48" s="101" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B49" s="46"/>
-      <c r="C49" s="54" t="s">
+      <c r="B49" s="83"/>
+      <c r="C49" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="D49" s="55"/>
-      <c r="E49" s="54" t="s">
+      <c r="D49" s="88"/>
+      <c r="E49" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="F49" s="55"/>
-      <c r="G49" s="54" t="s">
+      <c r="F49" s="88"/>
+      <c r="G49" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H49" s="55"/>
+      <c r="H49" s="88"/>
       <c r="I49" s="20"/>
-      <c r="J49" s="100" t="s">
+      <c r="J49" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="K49" s="101"/>
+      <c r="K49" s="100"/>
       <c r="M49" s="2"/>
-      <c r="N49" s="48" t="s">
+      <c r="N49" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="O49" s="49"/>
-      <c r="P49" s="99"/>
+      <c r="O49" s="76"/>
+      <c r="P49" s="101"/>
     </row>
     <row r="50" spans="1:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="B50" s="47"/>
+      <c r="B50" s="84"/>
       <c r="C50" s="1" t="s">
         <v>4</v>
       </c>
@@ -9103,47 +9103,47 @@
       </c>
     </row>
     <row r="93" spans="1:16" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="64" t="s">
+      <c r="B93" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C93" s="64"/>
-      <c r="D93" s="93" t="s">
+      <c r="C93" s="40"/>
+      <c r="D93" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="E93" s="93"/>
-      <c r="F93" s="93"/>
-      <c r="G93" s="93"/>
-      <c r="H93" s="93"/>
-      <c r="I93" s="93"/>
-      <c r="J93" s="93"/>
-      <c r="K93" s="93"/>
-      <c r="L93" s="93"/>
-      <c r="M93" s="93"/>
-      <c r="N93" s="93"/>
-      <c r="O93" s="93"/>
-      <c r="P93" s="93"/>
+      <c r="E93" s="94"/>
+      <c r="F93" s="94"/>
+      <c r="G93" s="94"/>
+      <c r="H93" s="94"/>
+      <c r="I93" s="94"/>
+      <c r="J93" s="94"/>
+      <c r="K93" s="94"/>
+      <c r="L93" s="94"/>
+      <c r="M93" s="94"/>
+      <c r="N93" s="94"/>
+      <c r="O93" s="94"/>
+      <c r="P93" s="94"/>
     </row>
     <row r="94" spans="1:16" ht="35.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B94" s="94" t="s">
+      <c r="B94" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="C94" s="94"/>
-      <c r="D94" s="94"/>
-      <c r="E94" s="94"/>
-      <c r="F94" s="94"/>
-      <c r="G94" s="94"/>
-      <c r="H94" s="94"/>
-      <c r="I94" s="94"/>
-      <c r="J94" s="94"/>
-      <c r="K94" s="94"/>
-      <c r="L94" s="94"/>
-      <c r="M94" s="94"/>
-      <c r="N94" s="94"/>
-      <c r="O94" s="94"/>
-      <c r="P94" s="94"/>
+      <c r="C94" s="93"/>
+      <c r="D94" s="93"/>
+      <c r="E94" s="93"/>
+      <c r="F94" s="93"/>
+      <c r="G94" s="93"/>
+      <c r="H94" s="93"/>
+      <c r="I94" s="93"/>
+      <c r="J94" s="93"/>
+      <c r="K94" s="93"/>
+      <c r="L94" s="93"/>
+      <c r="M94" s="93"/>
+      <c r="N94" s="93"/>
+      <c r="O94" s="93"/>
+      <c r="P94" s="93"/>
     </row>
     <row r="95" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B95" s="46" t="s">
+      <c r="B95" s="83" t="s">
         <v>28</v>
       </c>
       <c r="C95" s="95" t="s">
@@ -9168,38 +9168,38 @@
         <v>7</v>
       </c>
       <c r="O95" s="98"/>
-      <c r="P95" s="99" t="s">
+      <c r="P95" s="101" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="96" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B96" s="46"/>
-      <c r="C96" s="54" t="s">
+      <c r="B96" s="83"/>
+      <c r="C96" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="D96" s="55"/>
-      <c r="E96" s="54" t="s">
+      <c r="D96" s="88"/>
+      <c r="E96" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="F96" s="55"/>
-      <c r="G96" s="54" t="s">
+      <c r="F96" s="88"/>
+      <c r="G96" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H96" s="55"/>
+      <c r="H96" s="88"/>
       <c r="I96" s="20"/>
-      <c r="J96" s="100" t="s">
+      <c r="J96" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="K96" s="101"/>
+      <c r="K96" s="100"/>
       <c r="M96" s="2"/>
-      <c r="N96" s="48" t="s">
+      <c r="N96" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="O96" s="49"/>
-      <c r="P96" s="99"/>
+      <c r="O96" s="76"/>
+      <c r="P96" s="101"/>
     </row>
     <row r="97" spans="1:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="B97" s="47"/>
+      <c r="B97" s="84"/>
       <c r="C97" s="1" t="s">
         <v>4</v>
       </c>
@@ -10758,47 +10758,47 @@
       </c>
     </row>
     <row r="140" spans="1:16" ht="27.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B140" s="64" t="s">
+      <c r="B140" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C140" s="64"/>
-      <c r="D140" s="93" t="s">
+      <c r="C140" s="40"/>
+      <c r="D140" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="E140" s="93"/>
-      <c r="F140" s="93"/>
-      <c r="G140" s="93"/>
-      <c r="H140" s="93"/>
-      <c r="I140" s="93"/>
-      <c r="J140" s="93"/>
-      <c r="K140" s="93"/>
-      <c r="L140" s="93"/>
-      <c r="M140" s="93"/>
-      <c r="N140" s="93"/>
-      <c r="O140" s="93"/>
-      <c r="P140" s="93"/>
+      <c r="E140" s="94"/>
+      <c r="F140" s="94"/>
+      <c r="G140" s="94"/>
+      <c r="H140" s="94"/>
+      <c r="I140" s="94"/>
+      <c r="J140" s="94"/>
+      <c r="K140" s="94"/>
+      <c r="L140" s="94"/>
+      <c r="M140" s="94"/>
+      <c r="N140" s="94"/>
+      <c r="O140" s="94"/>
+      <c r="P140" s="94"/>
     </row>
     <row r="141" spans="1:16" ht="32.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B141" s="94" t="s">
+      <c r="B141" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="C141" s="94"/>
-      <c r="D141" s="94"/>
-      <c r="E141" s="94"/>
-      <c r="F141" s="94"/>
-      <c r="G141" s="94"/>
-      <c r="H141" s="94"/>
-      <c r="I141" s="94"/>
-      <c r="J141" s="94"/>
-      <c r="K141" s="94"/>
-      <c r="L141" s="94"/>
-      <c r="M141" s="94"/>
-      <c r="N141" s="94"/>
-      <c r="O141" s="94"/>
-      <c r="P141" s="94"/>
+      <c r="C141" s="93"/>
+      <c r="D141" s="93"/>
+      <c r="E141" s="93"/>
+      <c r="F141" s="93"/>
+      <c r="G141" s="93"/>
+      <c r="H141" s="93"/>
+      <c r="I141" s="93"/>
+      <c r="J141" s="93"/>
+      <c r="K141" s="93"/>
+      <c r="L141" s="93"/>
+      <c r="M141" s="93"/>
+      <c r="N141" s="93"/>
+      <c r="O141" s="93"/>
+      <c r="P141" s="93"/>
     </row>
     <row r="142" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B142" s="46" t="s">
+      <c r="B142" s="83" t="s">
         <v>28</v>
       </c>
       <c r="C142" s="95" t="s">
@@ -10823,38 +10823,38 @@
         <v>7</v>
       </c>
       <c r="O142" s="98"/>
-      <c r="P142" s="99" t="s">
+      <c r="P142" s="101" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="143" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B143" s="46"/>
-      <c r="C143" s="54" t="s">
+      <c r="B143" s="83"/>
+      <c r="C143" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="D143" s="55"/>
-      <c r="E143" s="54" t="s">
+      <c r="D143" s="88"/>
+      <c r="E143" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="F143" s="55"/>
-      <c r="G143" s="54" t="s">
+      <c r="F143" s="88"/>
+      <c r="G143" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H143" s="55"/>
+      <c r="H143" s="88"/>
       <c r="I143" s="20"/>
-      <c r="J143" s="100" t="s">
+      <c r="J143" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="K143" s="101"/>
+      <c r="K143" s="100"/>
       <c r="M143" s="2"/>
-      <c r="N143" s="48" t="s">
+      <c r="N143" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="O143" s="49"/>
-      <c r="P143" s="99"/>
+      <c r="O143" s="76"/>
+      <c r="P143" s="101"/>
     </row>
     <row r="144" spans="1:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="B144" s="47"/>
+      <c r="B144" s="84"/>
       <c r="C144" s="1" t="s">
         <v>4</v>
       </c>
@@ -12430,47 +12430,47 @@
     </row>
     <row r="185" spans="1:20" ht="25.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="187" spans="1:20" ht="21.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B187" s="64" t="s">
+      <c r="B187" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C187" s="64"/>
-      <c r="D187" s="93" t="s">
+      <c r="C187" s="40"/>
+      <c r="D187" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="E187" s="93"/>
-      <c r="F187" s="93"/>
-      <c r="G187" s="93"/>
-      <c r="H187" s="93"/>
-      <c r="I187" s="93"/>
-      <c r="J187" s="93"/>
-      <c r="K187" s="93"/>
-      <c r="L187" s="93"/>
-      <c r="M187" s="93"/>
-      <c r="N187" s="93"/>
-      <c r="O187" s="93"/>
-      <c r="P187" s="93"/>
+      <c r="E187" s="94"/>
+      <c r="F187" s="94"/>
+      <c r="G187" s="94"/>
+      <c r="H187" s="94"/>
+      <c r="I187" s="94"/>
+      <c r="J187" s="94"/>
+      <c r="K187" s="94"/>
+      <c r="L187" s="94"/>
+      <c r="M187" s="94"/>
+      <c r="N187" s="94"/>
+      <c r="O187" s="94"/>
+      <c r="P187" s="94"/>
     </row>
     <row r="188" spans="1:20" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B188" s="94" t="s">
+      <c r="B188" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="C188" s="94"/>
-      <c r="D188" s="94"/>
-      <c r="E188" s="94"/>
-      <c r="F188" s="94"/>
-      <c r="G188" s="94"/>
-      <c r="H188" s="94"/>
-      <c r="I188" s="94"/>
-      <c r="J188" s="94"/>
-      <c r="K188" s="94"/>
-      <c r="L188" s="94"/>
-      <c r="M188" s="94"/>
-      <c r="N188" s="94"/>
-      <c r="O188" s="94"/>
-      <c r="P188" s="94"/>
+      <c r="C188" s="93"/>
+      <c r="D188" s="93"/>
+      <c r="E188" s="93"/>
+      <c r="F188" s="93"/>
+      <c r="G188" s="93"/>
+      <c r="H188" s="93"/>
+      <c r="I188" s="93"/>
+      <c r="J188" s="93"/>
+      <c r="K188" s="93"/>
+      <c r="L188" s="93"/>
+      <c r="M188" s="93"/>
+      <c r="N188" s="93"/>
+      <c r="O188" s="93"/>
+      <c r="P188" s="93"/>
     </row>
     <row r="189" spans="1:20" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B189" s="46" t="s">
+      <c r="B189" s="83" t="s">
         <v>28</v>
       </c>
       <c r="C189" s="95" t="s">
@@ -12495,42 +12495,42 @@
         <v>7</v>
       </c>
       <c r="O189" s="98"/>
-      <c r="P189" s="99" t="s">
+      <c r="P189" s="101" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="190" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B190" s="46"/>
-      <c r="C190" s="54" t="s">
+      <c r="B190" s="83"/>
+      <c r="C190" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="D190" s="55"/>
-      <c r="E190" s="54" t="s">
+      <c r="D190" s="88"/>
+      <c r="E190" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="F190" s="55"/>
-      <c r="G190" s="54" t="s">
+      <c r="F190" s="88"/>
+      <c r="G190" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H190" s="55"/>
+      <c r="H190" s="88"/>
       <c r="I190" s="20"/>
-      <c r="J190" s="100" t="s">
+      <c r="J190" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="K190" s="101"/>
+      <c r="K190" s="100"/>
       <c r="M190" s="2"/>
-      <c r="N190" s="48" t="s">
+      <c r="N190" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="O190" s="49"/>
-      <c r="P190" s="99"/>
+      <c r="O190" s="76"/>
+      <c r="P190" s="101"/>
       <c r="Q190" s="2"/>
       <c r="R190" s="2"/>
       <c r="S190" s="2"/>
       <c r="T190" s="2"/>
     </row>
     <row r="191" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="B191" s="47"/>
+      <c r="B191" s="84"/>
       <c r="C191" s="1" t="s">
         <v>4</v>
       </c>
@@ -14217,47 +14217,47 @@
     <row r="227" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="228" spans="1:16" ht="23.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="230" spans="1:16" ht="24" x14ac:dyDescent="0.3">
-      <c r="B230" s="64" t="s">
+      <c r="B230" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C230" s="64"/>
-      <c r="D230" s="93" t="s">
+      <c r="C230" s="40"/>
+      <c r="D230" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="E230" s="93"/>
-      <c r="F230" s="93"/>
-      <c r="G230" s="93"/>
-      <c r="H230" s="93"/>
-      <c r="I230" s="93"/>
-      <c r="J230" s="93"/>
-      <c r="K230" s="93"/>
-      <c r="L230" s="93"/>
-      <c r="M230" s="93"/>
-      <c r="N230" s="93"/>
-      <c r="O230" s="93"/>
-      <c r="P230" s="93"/>
+      <c r="E230" s="94"/>
+      <c r="F230" s="94"/>
+      <c r="G230" s="94"/>
+      <c r="H230" s="94"/>
+      <c r="I230" s="94"/>
+      <c r="J230" s="94"/>
+      <c r="K230" s="94"/>
+      <c r="L230" s="94"/>
+      <c r="M230" s="94"/>
+      <c r="N230" s="94"/>
+      <c r="O230" s="94"/>
+      <c r="P230" s="94"/>
     </row>
     <row r="231" spans="1:16" ht="34.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B231" s="94" t="s">
+      <c r="B231" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="C231" s="94"/>
-      <c r="D231" s="94"/>
-      <c r="E231" s="94"/>
-      <c r="F231" s="94"/>
-      <c r="G231" s="94"/>
-      <c r="H231" s="94"/>
-      <c r="I231" s="94"/>
-      <c r="J231" s="94"/>
-      <c r="K231" s="94"/>
-      <c r="L231" s="94"/>
-      <c r="M231" s="94"/>
-      <c r="N231" s="94"/>
-      <c r="O231" s="94"/>
-      <c r="P231" s="94"/>
+      <c r="C231" s="93"/>
+      <c r="D231" s="93"/>
+      <c r="E231" s="93"/>
+      <c r="F231" s="93"/>
+      <c r="G231" s="93"/>
+      <c r="H231" s="93"/>
+      <c r="I231" s="93"/>
+      <c r="J231" s="93"/>
+      <c r="K231" s="93"/>
+      <c r="L231" s="93"/>
+      <c r="M231" s="93"/>
+      <c r="N231" s="93"/>
+      <c r="O231" s="93"/>
+      <c r="P231" s="93"/>
     </row>
     <row r="232" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B232" s="46" t="s">
+      <c r="B232" s="83" t="s">
         <v>28</v>
       </c>
       <c r="C232" s="95" t="s">
@@ -14282,38 +14282,38 @@
         <v>7</v>
       </c>
       <c r="O232" s="98"/>
-      <c r="P232" s="99" t="s">
+      <c r="P232" s="101" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="233" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B233" s="46"/>
-      <c r="C233" s="54" t="s">
+      <c r="B233" s="83"/>
+      <c r="C233" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="D233" s="55"/>
-      <c r="E233" s="54" t="s">
+      <c r="D233" s="88"/>
+      <c r="E233" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="F233" s="55"/>
-      <c r="G233" s="54" t="s">
+      <c r="F233" s="88"/>
+      <c r="G233" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H233" s="55"/>
+      <c r="H233" s="88"/>
       <c r="I233" s="20"/>
-      <c r="J233" s="100" t="s">
+      <c r="J233" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="K233" s="101"/>
+      <c r="K233" s="100"/>
       <c r="M233" s="2"/>
-      <c r="N233" s="48" t="s">
+      <c r="N233" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="O233" s="49"/>
-      <c r="P233" s="99"/>
+      <c r="O233" s="76"/>
+      <c r="P233" s="101"/>
     </row>
     <row r="234" spans="1:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="B234" s="47"/>
+      <c r="B234" s="84"/>
       <c r="C234" s="1" t="s">
         <v>4</v>
       </c>
@@ -16163,47 +16163,47 @@
     </row>
     <row r="276" spans="1:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="277" spans="1:16" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B277" s="64" t="s">
+      <c r="B277" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C277" s="64"/>
-      <c r="D277" s="93" t="s">
+      <c r="C277" s="40"/>
+      <c r="D277" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="E277" s="93"/>
-      <c r="F277" s="93"/>
-      <c r="G277" s="93"/>
-      <c r="H277" s="93"/>
-      <c r="I277" s="93"/>
-      <c r="J277" s="93"/>
-      <c r="K277" s="93"/>
-      <c r="L277" s="93"/>
-      <c r="M277" s="93"/>
-      <c r="N277" s="93"/>
-      <c r="O277" s="93"/>
-      <c r="P277" s="93"/>
+      <c r="E277" s="94"/>
+      <c r="F277" s="94"/>
+      <c r="G277" s="94"/>
+      <c r="H277" s="94"/>
+      <c r="I277" s="94"/>
+      <c r="J277" s="94"/>
+      <c r="K277" s="94"/>
+      <c r="L277" s="94"/>
+      <c r="M277" s="94"/>
+      <c r="N277" s="94"/>
+      <c r="O277" s="94"/>
+      <c r="P277" s="94"/>
     </row>
     <row r="278" spans="1:16" ht="28.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B278" s="94" t="s">
+      <c r="B278" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="C278" s="94"/>
-      <c r="D278" s="94"/>
-      <c r="E278" s="94"/>
-      <c r="F278" s="94"/>
-      <c r="G278" s="94"/>
-      <c r="H278" s="94"/>
-      <c r="I278" s="94"/>
-      <c r="J278" s="94"/>
-      <c r="K278" s="94"/>
-      <c r="L278" s="94"/>
-      <c r="M278" s="94"/>
-      <c r="N278" s="94"/>
-      <c r="O278" s="94"/>
-      <c r="P278" s="94"/>
+      <c r="C278" s="93"/>
+      <c r="D278" s="93"/>
+      <c r="E278" s="93"/>
+      <c r="F278" s="93"/>
+      <c r="G278" s="93"/>
+      <c r="H278" s="93"/>
+      <c r="I278" s="93"/>
+      <c r="J278" s="93"/>
+      <c r="K278" s="93"/>
+      <c r="L278" s="93"/>
+      <c r="M278" s="93"/>
+      <c r="N278" s="93"/>
+      <c r="O278" s="93"/>
+      <c r="P278" s="93"/>
     </row>
     <row r="279" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B279" s="46" t="s">
+      <c r="B279" s="83" t="s">
         <v>28</v>
       </c>
       <c r="C279" s="95" t="s">
@@ -16228,38 +16228,38 @@
         <v>7</v>
       </c>
       <c r="O279" s="98"/>
-      <c r="P279" s="99" t="s">
+      <c r="P279" s="101" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="280" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B280" s="46"/>
-      <c r="C280" s="54" t="s">
+      <c r="B280" s="83"/>
+      <c r="C280" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="D280" s="55"/>
-      <c r="E280" s="54" t="s">
+      <c r="D280" s="88"/>
+      <c r="E280" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="F280" s="55"/>
-      <c r="G280" s="54" t="s">
+      <c r="F280" s="88"/>
+      <c r="G280" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H280" s="55"/>
+      <c r="H280" s="88"/>
       <c r="I280" s="20"/>
-      <c r="J280" s="100" t="s">
+      <c r="J280" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="K280" s="101"/>
+      <c r="K280" s="100"/>
       <c r="M280" s="2"/>
-      <c r="N280" s="48" t="s">
+      <c r="N280" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="O280" s="49"/>
-      <c r="P280" s="99"/>
+      <c r="O280" s="76"/>
+      <c r="P280" s="101"/>
     </row>
     <row r="281" spans="1:16" ht="16" x14ac:dyDescent="0.2">
-      <c r="B281" s="47"/>
+      <c r="B281" s="84"/>
       <c r="C281" s="1" t="s">
         <v>4</v>
       </c>
@@ -17018,21 +17018,79 @@
     </row>
   </sheetData>
   <mergeCells count="105">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:P2"/>
-    <mergeCell ref="D1:P1"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="B277:C277"/>
+    <mergeCell ref="D277:P277"/>
+    <mergeCell ref="B278:P278"/>
+    <mergeCell ref="C279:D279"/>
+    <mergeCell ref="E279:F279"/>
+    <mergeCell ref="G279:H279"/>
+    <mergeCell ref="J279:K279"/>
+    <mergeCell ref="N279:O279"/>
+    <mergeCell ref="P279:P280"/>
+    <mergeCell ref="C280:D280"/>
+    <mergeCell ref="E280:F280"/>
+    <mergeCell ref="G280:H280"/>
+    <mergeCell ref="J280:K280"/>
+    <mergeCell ref="N280:O280"/>
+    <mergeCell ref="B279:B281"/>
+    <mergeCell ref="B231:P231"/>
+    <mergeCell ref="C232:D232"/>
+    <mergeCell ref="E232:F232"/>
+    <mergeCell ref="G232:H232"/>
+    <mergeCell ref="J232:K232"/>
+    <mergeCell ref="N232:O232"/>
+    <mergeCell ref="P232:P233"/>
+    <mergeCell ref="C233:D233"/>
+    <mergeCell ref="E233:F233"/>
+    <mergeCell ref="G233:H233"/>
+    <mergeCell ref="J233:K233"/>
+    <mergeCell ref="N233:O233"/>
+    <mergeCell ref="B232:B234"/>
+    <mergeCell ref="B230:C230"/>
+    <mergeCell ref="D230:P230"/>
+    <mergeCell ref="D187:P187"/>
+    <mergeCell ref="B188:P188"/>
+    <mergeCell ref="P189:P190"/>
+    <mergeCell ref="C189:D189"/>
+    <mergeCell ref="E189:F189"/>
+    <mergeCell ref="G189:H189"/>
+    <mergeCell ref="J189:K189"/>
+    <mergeCell ref="N189:O189"/>
+    <mergeCell ref="B187:C187"/>
+    <mergeCell ref="C190:D190"/>
+    <mergeCell ref="E190:F190"/>
+    <mergeCell ref="G190:H190"/>
+    <mergeCell ref="J190:K190"/>
+    <mergeCell ref="N190:O190"/>
+    <mergeCell ref="B189:B191"/>
+    <mergeCell ref="B141:P141"/>
+    <mergeCell ref="P142:P143"/>
+    <mergeCell ref="C143:D143"/>
+    <mergeCell ref="E143:F143"/>
+    <mergeCell ref="G143:H143"/>
+    <mergeCell ref="J143:K143"/>
+    <mergeCell ref="N143:O143"/>
+    <mergeCell ref="B142:B144"/>
+    <mergeCell ref="C142:D142"/>
+    <mergeCell ref="E142:F142"/>
+    <mergeCell ref="G142:H142"/>
+    <mergeCell ref="J142:K142"/>
+    <mergeCell ref="N142:O142"/>
+    <mergeCell ref="B140:C140"/>
+    <mergeCell ref="D140:P140"/>
+    <mergeCell ref="B94:P94"/>
+    <mergeCell ref="C95:D95"/>
+    <mergeCell ref="E95:F95"/>
+    <mergeCell ref="G95:H95"/>
+    <mergeCell ref="J95:K95"/>
+    <mergeCell ref="N95:O95"/>
+    <mergeCell ref="P95:P96"/>
+    <mergeCell ref="C96:D96"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="G96:H96"/>
+    <mergeCell ref="J96:K96"/>
+    <mergeCell ref="N96:O96"/>
+    <mergeCell ref="B95:B97"/>
     <mergeCell ref="G49:H49"/>
     <mergeCell ref="J49:K49"/>
     <mergeCell ref="N49:O49"/>
@@ -17050,81 +17108,23 @@
     <mergeCell ref="P48:P49"/>
     <mergeCell ref="C49:D49"/>
     <mergeCell ref="E49:F49"/>
-    <mergeCell ref="B140:C140"/>
-    <mergeCell ref="D140:P140"/>
-    <mergeCell ref="B94:P94"/>
-    <mergeCell ref="C95:D95"/>
-    <mergeCell ref="E95:F95"/>
-    <mergeCell ref="G95:H95"/>
-    <mergeCell ref="J95:K95"/>
-    <mergeCell ref="N95:O95"/>
-    <mergeCell ref="P95:P96"/>
-    <mergeCell ref="C96:D96"/>
-    <mergeCell ref="E96:F96"/>
-    <mergeCell ref="G96:H96"/>
-    <mergeCell ref="J96:K96"/>
-    <mergeCell ref="N96:O96"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="B141:P141"/>
-    <mergeCell ref="P142:P143"/>
-    <mergeCell ref="C143:D143"/>
-    <mergeCell ref="E143:F143"/>
-    <mergeCell ref="G143:H143"/>
-    <mergeCell ref="J143:K143"/>
-    <mergeCell ref="N143:O143"/>
-    <mergeCell ref="B142:B144"/>
-    <mergeCell ref="C142:D142"/>
-    <mergeCell ref="E142:F142"/>
-    <mergeCell ref="G142:H142"/>
-    <mergeCell ref="J142:K142"/>
-    <mergeCell ref="N142:O142"/>
-    <mergeCell ref="B230:C230"/>
-    <mergeCell ref="D230:P230"/>
-    <mergeCell ref="D187:P187"/>
-    <mergeCell ref="B188:P188"/>
-    <mergeCell ref="P189:P190"/>
-    <mergeCell ref="C189:D189"/>
-    <mergeCell ref="E189:F189"/>
-    <mergeCell ref="G189:H189"/>
-    <mergeCell ref="J189:K189"/>
-    <mergeCell ref="N189:O189"/>
-    <mergeCell ref="B187:C187"/>
-    <mergeCell ref="C190:D190"/>
-    <mergeCell ref="E190:F190"/>
-    <mergeCell ref="G190:H190"/>
-    <mergeCell ref="J190:K190"/>
-    <mergeCell ref="N190:O190"/>
-    <mergeCell ref="B189:B191"/>
-    <mergeCell ref="B231:P231"/>
-    <mergeCell ref="C232:D232"/>
-    <mergeCell ref="E232:F232"/>
-    <mergeCell ref="G232:H232"/>
-    <mergeCell ref="J232:K232"/>
-    <mergeCell ref="N232:O232"/>
-    <mergeCell ref="P232:P233"/>
-    <mergeCell ref="C233:D233"/>
-    <mergeCell ref="E233:F233"/>
-    <mergeCell ref="G233:H233"/>
-    <mergeCell ref="J233:K233"/>
-    <mergeCell ref="N233:O233"/>
-    <mergeCell ref="B232:B234"/>
-    <mergeCell ref="B277:C277"/>
-    <mergeCell ref="D277:P277"/>
-    <mergeCell ref="B278:P278"/>
-    <mergeCell ref="C279:D279"/>
-    <mergeCell ref="E279:F279"/>
-    <mergeCell ref="G279:H279"/>
-    <mergeCell ref="J279:K279"/>
-    <mergeCell ref="N279:O279"/>
-    <mergeCell ref="P279:P280"/>
-    <mergeCell ref="C280:D280"/>
-    <mergeCell ref="E280:F280"/>
-    <mergeCell ref="G280:H280"/>
-    <mergeCell ref="J280:K280"/>
-    <mergeCell ref="N280:O280"/>
-    <mergeCell ref="B279:B281"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="D1:P1"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P3:P4"/>
   </mergeCells>
-  <conditionalFormatting sqref="P3 P5:P42 P48 P50:P89 P95 P97:P136 P142 P144:P183 P189 P232 P234:P273 P279 P281:P301 P191:P226">
+  <conditionalFormatting sqref="P3 P5:P42 P48 P50:P89 P95 P97:P136 P142 P144:P183 P189 P191:P226 P232 P234:P273 P279 P281:P301">
     <cfRule type="containsText" dxfId="0" priority="7" operator="containsText" text="Ja">
       <formula>NOT(ISERROR(SEARCH("Ja",P3)))</formula>
     </cfRule>

</xml_diff>